<commit_message>
Thanh toan ho so tot nghiep
</commit_message>
<xml_diff>
--- a/static/samples/Data_KhoaLuanTotNghiep.xlsx
+++ b/static/samples/Data_KhoaLuanTotNghiep.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\hienlth.io.vn\FIT_Tools\tools\static\samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74E3F213-ACB3-41B4-870A-71EE6C0B30D8}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CA9A1F2-8628-40FA-96C5-C651FFC97165}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,6 +22,112 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>ADMIN</author>
+  </authors>
+  <commentList>
+    <comment ref="D2" authorId="0" shapeId="0" xr:uid="{4110A04B-34DC-4B24-8E66-06F948A3D8C9}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>ADMIN:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Đơn giá 800k/khóa luận, tối đa 5 khóa luận/năm</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E2" authorId="0" shapeId="0" xr:uid="{B13F15E7-275B-46ED-B7C2-7214BB864B57}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>ADMIN:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+giá 150k/hội đồng</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F2" authorId="0" shapeId="0" xr:uid="{2A588199-F839-44AD-A703-5BA6EBE02EFD}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>ADMIN:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+giá 200k/khóa luận, bao gồm tiền hội đồng</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G2" authorId="0" shapeId="0" xr:uid="{F983118B-E15C-4812-8F6C-32EE6C309F24}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>ADMIN:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+giá 120k/hội đồng</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -85,7 +191,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -140,6 +246,19 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -433,7 +552,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -5416,5 +5535,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>